<commit_message>
Synchronize Round 10 figures and supplementary release
</commit_message>
<xml_diff>
--- a/tables/supplementary/Supplementary_Tables.xlsx
+++ b/tables/supplementary/Supplementary_Tables.xlsx
@@ -2,26 +2,26 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R47a2de354cc649d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S1" sheetId="2" r:id="Rd7e69776027c4656"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S2" sheetId="3" r:id="Re27788dd7ea74291"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S3" sheetId="4" r:id="R251a782ee4ac436e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S4" sheetId="5" r:id="Rd89b605486a84b0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S5" sheetId="6" r:id="Rf1952102e4854b81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S6" sheetId="7" r:id="Rc9a700771f68404e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S7" sheetId="8" r:id="R9c42c981f3d64c53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S8" sheetId="9" r:id="Rb132312a576042cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S9" sheetId="10" r:id="R7be36deb578941d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S10" sheetId="11" r:id="Rbaeb3e7c90da48a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S11" sheetId="12" r:id="R1da2102d288e4195"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S12" sheetId="13" r:id="R14b39b006eca4ce9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S13" sheetId="14" r:id="R2b36a0c77e804af3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S14" sheetId="15" r:id="Rde9cc72880324b20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S15" sheetId="16" r:id="Rc9c83deafa2d4a44"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S16" sheetId="17" r:id="Re0f5fa8f396a4d03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S17" sheetId="18" r:id="R33d7e97404b54d89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S18" sheetId="19" r:id="Rda976c07c8ae4e26"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S19" sheetId="20" r:id="Rd09d802a86644965"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R344ef5cf883d4ab2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S1" sheetId="2" r:id="R69529994e34948a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S2" sheetId="3" r:id="Rff90a0a140444314"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S3" sheetId="4" r:id="Rf14dbd0cc85e4e05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S4" sheetId="5" r:id="R717eb4d2a8f04080"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S5" sheetId="6" r:id="R9a596a83f5e64e22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S6" sheetId="7" r:id="Rafddccf72b044b02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S7" sheetId="8" r:id="Rdaa5df339a024982"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S8" sheetId="9" r:id="R0a2a342cc00b411f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S9" sheetId="10" r:id="R221ee685d0cd4b7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S10" sheetId="11" r:id="R05e81fed83e141b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S11" sheetId="12" r:id="R35faf259a54b4ed7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S12" sheetId="13" r:id="Rd441a13c7d3e4ced"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S13" sheetId="14" r:id="Rc1c662d120114646"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S14" sheetId="15" r:id="Reabe22ce2ccc4fc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S15" sheetId="16" r:id="R9d936273c4494693"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S16" sheetId="17" r:id="Rf0a1bb781c264c36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S17" sheetId="18" r:id="R1197bca4c98c45d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S18" sheetId="19" r:id="Rab0ea600c36a4101"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table S19" sheetId="20" r:id="R6309b72e81ee434a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -430,7 +430,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
-        <x:v>Local Alzheimer disease-cholesterol colocalization converges on TSPAN14 canonical-cryptic splice choice</x:v>
+        <x:v>A non-APOE Alzheimer disease-cholesterol locus converges on TSPAN14 splice choice</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -12062,7 +12062,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="F6" s="23" t="str">
-        <x:v>Cross-region bulk replication</x:v>
+        <x:v>Cross-tissue consistency in partially overlapping bulk neural tissues</x:v>
       </x:c>
       <x:c r="G6" s="23"/>
       <x:c r="H6" s="23"/>
@@ -65540,7 +65540,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="27.420000076293945" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="30" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="11.020000457763672" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="10" hidden="0" customWidth="1"/>
@@ -65740,7 +65740,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B5" s="23" t="str">
         <x:v>rs1870140</x:v>
@@ -65803,7 +65803,7 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
         <x:v>rs1870140</x:v>
@@ -65866,7 +65866,7 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B7" s="23" t="str">
         <x:v>rs1870140</x:v>
@@ -65929,7 +65929,7 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B8" s="23" t="str">
         <x:v>rs1870140</x:v>
@@ -65992,7 +65992,7 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B9" s="23" t="str">
         <x:v>rs6586028</x:v>
@@ -66055,7 +66055,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B10" s="23" t="str">
         <x:v>rs6586028</x:v>
@@ -66118,7 +66118,7 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B11" s="23" t="str">
         <x:v>rs6586028</x:v>
@@ -66181,7 +66181,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B12" s="23" t="str">
         <x:v>rs6586028</x:v>
@@ -66244,7 +66244,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B13" s="23" t="str">
         <x:v>rs1902660</x:v>
@@ -66307,7 +66307,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B14" s="23" t="str">
         <x:v>rs1902660</x:v>
@@ -66370,7 +66370,7 @@
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B15" s="23" t="str">
         <x:v>rs1902660</x:v>
@@ -66433,7 +66433,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B16" s="23" t="str">
         <x:v>rs1902660</x:v>
@@ -66496,7 +66496,7 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B17" s="23" t="str">
         <x:v>rs7080009</x:v>
@@ -66559,7 +66559,7 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B18" s="23" t="str">
         <x:v>rs7080009</x:v>
@@ -66622,7 +66622,7 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B19" s="23" t="str">
         <x:v>rs7080009</x:v>
@@ -66685,7 +66685,7 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B20" s="23" t="str">
         <x:v>rs7080009</x:v>
@@ -66748,7 +66748,7 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B21" s="23" t="str">
         <x:v>rs1870138</x:v>
@@ -66811,7 +66811,7 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B22" s="23" t="str">
         <x:v>rs1870138</x:v>
@@ -66874,7 +66874,7 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B23" s="23" t="str">
         <x:v>rs1870138</x:v>
@@ -66937,7 +66937,7 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B24" s="23" t="str">
         <x:v>rs1870138</x:v>
@@ -67000,7 +67000,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B25" s="23" t="str">
         <x:v>rs1870137</x:v>
@@ -67063,7 +67063,7 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B26" s="23" t="str">
         <x:v>rs1870137</x:v>
@@ -67126,7 +67126,7 @@
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B27" s="23" t="str">
         <x:v>rs1870137</x:v>
@@ -67189,7 +67189,7 @@
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="23" t="str">
-        <x:v>risk-aligned replication</x:v>
+        <x:v>risk-aligned cross-tissue consistency</x:v>
       </x:c>
       <x:c r="B28" s="23" t="str">
         <x:v>rs1870137</x:v>

</xml_diff>